<commit_message>
docs(cadrage): mise a jour du release planning
</commit_message>
<xml_diff>
--- a/docs/cadrage/equipe-6-release-planning.xlsx
+++ b/docs/cadrage/equipe-6-release-planning.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Windows11\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\woye\APOCALIPSSI\IPSSI_APOCAL_KIT\docs\cadrage\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F6A8937-EF35-4594-8455-4F66CAD42E51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D54F5441-E3B7-4DEB-9716-817D94F82FC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="118">
   <si>
     <t>APOCAL'IPSSI 2026 — EduTutor IA</t>
   </si>
@@ -78,9 +78,6 @@
     <t>Dépôt GitHub</t>
   </si>
   <si>
-    <t>/docs/cadrage/equipe-XX-release-planning.xlsx</t>
-  </si>
-  <si>
     <t>💡 Objectif de cet artefact</t>
   </si>
   <si>
@@ -375,41 +372,23 @@
     <t>Indicative seulement (pas de ratio fixe imposé) — à affiner avec le Product Backlog une fois les stories estimées en points.</t>
   </si>
   <si>
-    <t>À faire avant de commiter</t>
-  </si>
-  <si>
-    <t>☐</t>
-  </si>
-  <si>
-    <t>Remplacer les US-XX par les identifiants réels une fois la Story Map / Product Backlog validés par le PO.</t>
-  </si>
-  <si>
-    <t>Faire valider ce planning par le PO (animateur) avant 13h00.</t>
-  </si>
-  <si>
-    <t>Renommer le fichier : equipe-XX-release-planning.xlsx</t>
-  </si>
-  <si>
-    <t>Déposer dans /docs/cadrage/ du repo équipe et committer (message clair, type chore/docs).</t>
-  </si>
-  <si>
-    <t>Mettre à jour la feuille Burnup global à la fin de chaque sprint (colonne SP livrés).</t>
-  </si>
-  <si>
     <t>Équipe 6</t>
   </si>
   <si>
     <t>RAYAN ZEBAZE</t>
   </si>
   <si>
-    <t>RAYAN ZEBAZE &amp; vos noms</t>
+    <t>/docs/cadrage/equipe-6-release-planning.xlsx</t>
+  </si>
+  <si>
+    <t>RAYAN ZEBAZE, Hugo RAGUIN, Kahil MOKHTARI, Amine HADDANE, Souleymane FALL, Nikola MILOSAVLJEVIC, Dina CHAOUKI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -538,11 +517,6 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Arial"/>
-      <charset val="1"/>
-    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -651,31 +625,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -786,9 +737,29 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1776,149 +1747,149 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="41" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="9"/>
+      <c r="C2" s="41"/>
     </row>
     <row r="3" spans="2:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="8"/>
+      <c r="C3" s="42"/>
     </row>
     <row r="4" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="7"/>
+      <c r="C4" s="43"/>
     </row>
     <row r="6" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="6"/>
+      <c r="C6" s="40"/>
     </row>
     <row r="7" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="10" t="s">
+    <row r="8" spans="2:3" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="11" t="s">
-        <v>124</v>
+      <c r="C8" s="2" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="9" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="11" t="s">
-        <v>123</v>
+      <c r="C9" s="2" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="11" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="12" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="13" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="14" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B16" s="40" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="16" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B16" s="6" t="s">
+      <c r="C16" s="40"/>
+    </row>
+    <row r="17" spans="2:3" ht="90" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="6"/>
-    </row>
-    <row r="17" spans="2:3" ht="90" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="39"/>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B18" s="39"/>
+      <c r="C18" s="39"/>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B19" s="39"/>
+      <c r="C19" s="39"/>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B20" s="39"/>
+      <c r="C20" s="39"/>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B21" s="39"/>
+      <c r="C21" s="39"/>
+    </row>
+    <row r="23" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B23" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="5"/>
-    </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-    </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-    </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-    </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-    </row>
-    <row r="23" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B23" s="6" t="s">
+      <c r="C23" s="40"/>
+    </row>
+    <row r="24" spans="2:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="6"/>
-    </row>
-    <row r="24" spans="2:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="10" t="s">
+      <c r="C24" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C24" s="11" t="s">
+    </row>
+    <row r="25" spans="2:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="25" spans="2:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="10" t="s">
+      <c r="C25" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C25" s="11" t="s">
+    </row>
+    <row r="26" spans="2:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="26" spans="2:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="10" t="s">
+      <c r="C26" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="C26" s="11" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -1942,7 +1913,8 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="4" width="16" customWidth="1"/>
+    <col min="2" max="2" width="21.44140625" customWidth="1"/>
+    <col min="3" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="38" customWidth="1"/>
     <col min="6" max="6" width="30" customWidth="1"/>
     <col min="7" max="7" width="26" customWidth="1"/>
@@ -1950,306 +1922,306 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="44" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+    </row>
+    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="45" t="s">
+        <v>114</v>
+      </c>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+    </row>
+    <row r="4" spans="1:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-    </row>
-    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-    </row>
-    <row r="4" spans="1:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
+      <c r="B4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="C4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="D4" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="E4" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="F4" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="G4" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="H4" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="H4" s="12" t="s">
+    </row>
+    <row r="5" spans="1:8" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="13" t="s">
+      <c r="B5" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="C5" s="6">
+        <v>28</v>
+      </c>
+      <c r="D5" s="6">
+        <v>14</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="15">
+      <c r="F5" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="11">
         <v>28</v>
       </c>
-      <c r="D5" s="15">
-        <v>14</v>
-      </c>
-      <c r="E5" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="F5" s="16" t="s">
+      <c r="D6" s="11">
+        <v>18</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="H6" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="G5" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="H5" s="17" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="C6" s="20">
+    </row>
+    <row r="7" spans="1:8" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="6">
         <v>28</v>
       </c>
-      <c r="D6" s="20">
+      <c r="D7" s="6">
+        <v>20</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" s="11">
+        <v>28</v>
+      </c>
+      <c r="D8" s="11">
+        <v>20</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="G8" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="18">
+        <v>24</v>
+      </c>
+      <c r="D9" s="18">
+        <v>22</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="F9" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="H9" s="21" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="11">
+        <v>28</v>
+      </c>
+      <c r="D10" s="11">
         <v>18</v>
       </c>
-      <c r="E6" s="21" t="s">
-        <v>43</v>
-      </c>
-      <c r="F6" s="21" t="s">
-        <v>44</v>
-      </c>
-      <c r="G6" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="H6" s="23" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="C7" s="15">
-        <v>28</v>
-      </c>
-      <c r="D7" s="15">
+      <c r="E10" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="G10" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="H10" s="14" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="24">
+        <v>24</v>
+      </c>
+      <c r="D11" s="24">
+        <v>18</v>
+      </c>
+      <c r="E11" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="F11" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="G11" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="H11" s="26" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="27" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" s="29">
         <v>20</v>
       </c>
-      <c r="E7" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="F7" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="G7" s="24" t="s">
-        <v>50</v>
-      </c>
-      <c r="H7" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="20">
-        <v>28</v>
-      </c>
-      <c r="D8" s="20">
-        <v>20</v>
-      </c>
-      <c r="E8" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="F8" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="G8" s="22" t="s">
-        <v>55</v>
-      </c>
-      <c r="H8" s="23" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="25" t="s">
-        <v>56</v>
-      </c>
-      <c r="B9" s="26" t="s">
-        <v>57</v>
-      </c>
-      <c r="C9" s="27">
-        <v>24</v>
-      </c>
-      <c r="D9" s="27">
-        <v>22</v>
-      </c>
-      <c r="E9" s="28" t="s">
-        <v>58</v>
-      </c>
-      <c r="F9" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="G9" s="29" t="s">
-        <v>60</v>
-      </c>
-      <c r="H9" s="30" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="B10" s="19" t="s">
-        <v>63</v>
-      </c>
-      <c r="C10" s="20">
-        <v>28</v>
-      </c>
-      <c r="D10" s="20">
-        <v>18</v>
-      </c>
-      <c r="E10" s="21" t="s">
-        <v>64</v>
-      </c>
-      <c r="F10" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="G10" s="22" t="s">
-        <v>66</v>
-      </c>
-      <c r="H10" s="23" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="31" t="s">
-        <v>67</v>
-      </c>
-      <c r="B11" s="32" t="s">
-        <v>68</v>
-      </c>
-      <c r="C11" s="33">
-        <v>24</v>
-      </c>
-      <c r="D11" s="33">
-        <v>18</v>
-      </c>
-      <c r="E11" s="34" t="s">
-        <v>69</v>
-      </c>
-      <c r="F11" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="G11" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="H11" s="35" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="36" t="s">
-        <v>72</v>
-      </c>
-      <c r="B12" s="37" t="s">
+      <c r="D12" s="29">
+        <v>10</v>
+      </c>
+      <c r="E12" s="30" t="s">
         <v>73</v>
       </c>
-      <c r="C12" s="38">
-        <v>20</v>
-      </c>
-      <c r="D12" s="38">
-        <v>10</v>
-      </c>
-      <c r="E12" s="39" t="s">
+      <c r="F12" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="F12" s="39" t="s">
+      <c r="G12" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="H12" s="31" t="s">
         <v>75</v>
       </c>
-      <c r="G12" s="39" t="s">
-        <v>39</v>
-      </c>
-      <c r="H12" s="40" t="s">
+    </row>
+    <row r="13" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="32" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="41" t="s">
+      <c r="B13" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="B13" s="42" t="s">
-        <v>78</v>
-      </c>
-      <c r="C13" s="41">
+      <c r="C13" s="32">
         <f>SUM(C5:C12)</f>
         <v>208</v>
       </c>
-      <c r="D13" s="41">
+      <c r="D13" s="32">
         <f>SUM(D5:D12)</f>
         <v>140</v>
       </c>
-      <c r="E13" s="43"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="43"/>
-      <c r="H13" s="43"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="34"/>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="46" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" s="46"/>
+      <c r="C15" s="46"/>
+      <c r="D15" s="46"/>
+      <c r="E15" s="46"/>
+      <c r="F15" s="46"/>
+      <c r="G15" s="46"/>
+      <c r="H15" s="46"/>
+    </row>
+    <row r="16" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="46" t="s">
         <v>79</v>
       </c>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-    </row>
-    <row r="16" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
+      <c r="B16" s="46"/>
+      <c r="C16" s="46"/>
+      <c r="D16" s="46"/>
+      <c r="E16" s="46"/>
+      <c r="F16" s="46"/>
+      <c r="G16" s="46"/>
+      <c r="H16" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2274,252 +2246,252 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="44" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+    </row>
+    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="45" t="s">
         <v>81</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+    </row>
+    <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-    </row>
-    <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="12" t="s">
+      <c r="D4" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="E4" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="F4" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="G4" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="G4" s="12" t="s">
+    </row>
+    <row r="5" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="35" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="36" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="44" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" s="45" t="s">
-        <v>88</v>
-      </c>
-      <c r="C5" s="45">
+      <c r="C5" s="36">
         <v>14</v>
       </c>
-      <c r="D5" s="45">
+      <c r="D5" s="36">
         <v>0</v>
       </c>
-      <c r="E5" s="45">
+      <c r="E5" s="36">
         <f t="shared" ref="E5:E12" si="0">$C$12</f>
         <v>140</v>
       </c>
-      <c r="F5" s="45">
+      <c r="F5" s="36">
         <f t="shared" ref="F5:F12" si="1">D5-C5</f>
         <v>-14</v>
       </c>
-      <c r="G5" s="45" t="s">
+      <c r="G5" s="36" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="37" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="46" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" s="47" t="s">
-        <v>89</v>
-      </c>
-      <c r="C6" s="47">
+      <c r="B6" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" s="38">
         <v>32</v>
       </c>
-      <c r="D6" s="47">
+      <c r="D6" s="38">
         <v>0</v>
       </c>
-      <c r="E6" s="47">
+      <c r="E6" s="38">
         <f t="shared" si="0"/>
         <v>140</v>
       </c>
-      <c r="F6" s="47">
+      <c r="F6" s="38">
         <f t="shared" si="1"/>
         <v>-32</v>
       </c>
-      <c r="G6" s="47"/>
+      <c r="G6" s="38"/>
     </row>
     <row r="7" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="44" t="s">
-        <v>46</v>
-      </c>
-      <c r="B7" s="45" t="s">
-        <v>89</v>
-      </c>
-      <c r="C7" s="45">
+      <c r="A7" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="C7" s="36">
         <v>52</v>
       </c>
-      <c r="D7" s="45">
+      <c r="D7" s="36">
         <v>0</v>
       </c>
-      <c r="E7" s="45">
+      <c r="E7" s="36">
         <f t="shared" si="0"/>
         <v>140</v>
       </c>
-      <c r="F7" s="45">
+      <c r="F7" s="36">
         <f t="shared" si="1"/>
         <v>-52</v>
       </c>
-      <c r="G7" s="45"/>
+      <c r="G7" s="36"/>
     </row>
     <row r="8" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="46" t="s">
-        <v>51</v>
-      </c>
-      <c r="B8" s="47" t="s">
-        <v>90</v>
-      </c>
-      <c r="C8" s="47">
+      <c r="A8" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" s="38" t="s">
+        <v>89</v>
+      </c>
+      <c r="C8" s="38">
         <v>72</v>
       </c>
-      <c r="D8" s="47">
+      <c r="D8" s="38">
         <v>0</v>
       </c>
-      <c r="E8" s="47">
+      <c r="E8" s="38">
         <f t="shared" si="0"/>
         <v>140</v>
       </c>
-      <c r="F8" s="47">
+      <c r="F8" s="38">
         <f t="shared" si="1"/>
         <v>-72</v>
       </c>
-      <c r="G8" s="47"/>
+      <c r="G8" s="38"/>
     </row>
     <row r="9" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="44" t="s">
-        <v>56</v>
-      </c>
-      <c r="B9" s="45" t="s">
-        <v>90</v>
-      </c>
-      <c r="C9" s="45">
+      <c r="A9" s="35" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="36" t="s">
+        <v>89</v>
+      </c>
+      <c r="C9" s="36">
         <v>94</v>
       </c>
-      <c r="D9" s="45">
+      <c r="D9" s="36">
         <v>0</v>
       </c>
-      <c r="E9" s="45">
+      <c r="E9" s="36">
         <f t="shared" si="0"/>
         <v>140</v>
       </c>
-      <c r="F9" s="45">
+      <c r="F9" s="36">
         <f t="shared" si="1"/>
         <v>-94</v>
       </c>
-      <c r="G9" s="45" t="s">
+      <c r="G9" s="36" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="37" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="46" t="s">
-        <v>62</v>
-      </c>
-      <c r="B10" s="47" t="s">
-        <v>91</v>
-      </c>
-      <c r="C10" s="47">
+      <c r="B10" s="38" t="s">
+        <v>90</v>
+      </c>
+      <c r="C10" s="38">
         <v>112</v>
       </c>
-      <c r="D10" s="47">
+      <c r="D10" s="38">
         <v>0</v>
       </c>
-      <c r="E10" s="47">
+      <c r="E10" s="38">
         <f t="shared" si="0"/>
         <v>140</v>
       </c>
-      <c r="F10" s="47">
+      <c r="F10" s="38">
         <f t="shared" si="1"/>
         <v>-112</v>
       </c>
-      <c r="G10" s="47"/>
+      <c r="G10" s="38"/>
     </row>
     <row r="11" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="44" t="s">
-        <v>67</v>
-      </c>
-      <c r="B11" s="45" t="s">
-        <v>91</v>
-      </c>
-      <c r="C11" s="45">
+      <c r="A11" s="35" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="36" t="s">
+        <v>90</v>
+      </c>
+      <c r="C11" s="36">
         <v>130</v>
       </c>
-      <c r="D11" s="45">
+      <c r="D11" s="36">
         <v>0</v>
       </c>
-      <c r="E11" s="45">
+      <c r="E11" s="36">
         <f t="shared" si="0"/>
         <v>140</v>
       </c>
-      <c r="F11" s="45">
+      <c r="F11" s="36">
         <f t="shared" si="1"/>
         <v>-130</v>
       </c>
-      <c r="G11" s="45" t="s">
+      <c r="G11" s="36" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="37" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="46" t="s">
-        <v>72</v>
-      </c>
-      <c r="B12" s="47" t="s">
-        <v>92</v>
-      </c>
-      <c r="C12" s="47">
+      <c r="B12" s="38" t="s">
+        <v>91</v>
+      </c>
+      <c r="C12" s="38">
         <v>140</v>
       </c>
-      <c r="D12" s="47">
+      <c r="D12" s="38">
         <v>0</v>
       </c>
-      <c r="E12" s="47">
+      <c r="E12" s="38">
         <f t="shared" si="0"/>
         <v>140</v>
       </c>
-      <c r="F12" s="47">
+      <c r="F12" s="38">
         <f t="shared" si="1"/>
         <v>-140</v>
       </c>
-      <c r="G12" s="47" t="s">
-        <v>76</v>
+      <c r="G12" s="38" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
+      <c r="A14" s="46" t="s">
+        <v>92</v>
+      </c>
+      <c r="B14" s="46"/>
+      <c r="C14" s="46"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="46"/>
+      <c r="G14" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2543,147 +2515,105 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="44" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="44"/>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="47" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="4"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="B3" s="47"/>
+    </row>
+    <row r="4" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B3" s="1"/>
-    </row>
-    <row r="4" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+      <c r="B4" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B4" s="11" t="s">
+    </row>
+    <row r="5" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="10" t="s">
+      <c r="B5" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B5" s="11" t="s">
+    </row>
+    <row r="6" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+      <c r="B6" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B6" s="11" t="s">
+    </row>
+    <row r="7" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="10" t="s">
+      <c r="B7" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B7" s="11" t="s">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="47" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="B9" s="47"/>
+    </row>
+    <row r="10" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="B9" s="1"/>
-    </row>
-    <row r="10" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="10" t="s">
+      <c r="B10" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B10" s="11" t="s">
+    </row>
+    <row r="11" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="10" t="s">
+      <c r="B11" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B11" s="11" t="s">
+    </row>
+    <row r="12" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="10" t="s">
+      <c r="B12" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B12" s="11" t="s">
+    </row>
+    <row r="13" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="10" t="s">
+      <c r="B13" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B13" s="11" t="s">
+    </row>
+    <row r="14" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="10" t="s">
+      <c r="B14" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B14" s="11" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="B16" s="1"/>
-    </row>
-    <row r="17" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="48" t="s">
-        <v>116</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="48" t="s">
-        <v>116</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="48" t="s">
-        <v>116</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="48" t="s">
-        <v>116</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="48" t="s">
-        <v>116</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>121</v>
-      </c>
-    </row>
+    </row>
+    <row r="17" ht="24" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="18" ht="24" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="19" ht="24" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="20" ht="24" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="21" ht="24" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A16:B16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>